<commit_message>
altera o nome do metodo no arquivo que rodou a simulacao e no resultado mais recente 20250418 o desvio padrao para RMSE
</commit_message>
<xml_diff>
--- a/202505_resultados/ 2012 _tabela_n_miss.xlsx
+++ b/202505_resultados/ 2012 _tabela_n_miss.xlsx
@@ -23,10 +23,10 @@
     <t xml:space="preserve">Estado civil da mãe</t>
   </si>
   <si>
-    <t xml:space="preserve">Turno do nascimento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de função do responsável pelo preenchimento da DN</t>
+    <t xml:space="preserve">Turno da hora do nascimento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idade da mãe</t>
   </si>
   <si>
     <t xml:space="preserve">RO</t>

</xml_diff>